<commit_message>
Update forecast & dashboard 2026-06-18
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrohfm/Downloads/world-cup-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1167DB86-0018-154F-9FE7-38255F6D96AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C8810E-FFD1-1746-840C-23904DD4AED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6880" yWindow="2880" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -1732,12 +1732,16 @@
       <c r="D25" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
+      <c r="E25" s="5">
+        <v>1</v>
+      </c>
+      <c r="F25" s="5">
+        <v>1</v>
+      </c>
       <c r="G25" s="5"/>
       <c r="H25" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -1753,12 +1757,16 @@
       <c r="D26" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
+      <c r="E26" s="5">
+        <v>4</v>
+      </c>
+      <c r="F26" s="5">
+        <v>2</v>
+      </c>
       <c r="G26" s="5"/>
       <c r="H26" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -1774,12 +1782,16 @@
       <c r="D27" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
+      <c r="E27" s="5">
+        <v>1</v>
+      </c>
+      <c r="F27" s="5">
+        <v>0</v>
+      </c>
       <c r="G27" s="5"/>
       <c r="H27" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -1795,12 +1807,16 @@
       <c r="D28" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
+      <c r="E28" s="5">
+        <v>1</v>
+      </c>
+      <c r="F28" s="5">
+        <v>3</v>
+      </c>
       <c r="G28" s="5"/>
       <c r="H28" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update forecast & dashboard 2026-06-19
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrohfm/Downloads/world-cup-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C8810E-FFD1-1746-840C-23904DD4AED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C8067B-BF04-DF4A-81C8-A680067D5C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6880" yWindow="2880" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1832,12 +1832,16 @@
       <c r="D29" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
+      <c r="E29" s="5">
+        <v>1</v>
+      </c>
+      <c r="F29" s="5">
+        <v>1</v>
+      </c>
       <c r="G29" s="5"/>
       <c r="H29" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
@@ -1853,12 +1857,16 @@
       <c r="D30" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
+      <c r="E30" s="5">
+        <v>4</v>
+      </c>
+      <c r="F30" s="5">
+        <v>1</v>
+      </c>
       <c r="G30" s="5"/>
       <c r="H30" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
@@ -1874,12 +1882,16 @@
       <c r="D31" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
+      <c r="E31" s="5">
+        <v>6</v>
+      </c>
+      <c r="F31" s="5">
+        <v>0</v>
+      </c>
       <c r="G31" s="5"/>
       <c r="H31" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
@@ -1895,12 +1907,16 @@
       <c r="D32" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
+      <c r="E32" s="5">
+        <v>1</v>
+      </c>
+      <c r="F32" s="5">
+        <v>0</v>
+      </c>
       <c r="G32" s="5"/>
       <c r="H32" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update forecast & dashboard 2026-06-20
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrohfm/Downloads/world-cup-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C8067B-BF04-DF4A-81C8-A680067D5C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1747791C-AC36-604C-A77D-A309E88A70E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6880" yWindow="2880" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1932,12 +1932,16 @@
       <c r="D33" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
+      <c r="E33" s="5">
+        <v>2</v>
+      </c>
+      <c r="F33" s="5">
+        <v>0</v>
+      </c>
       <c r="G33" s="5"/>
       <c r="H33" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
@@ -1953,12 +1957,16 @@
       <c r="D34" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
+      <c r="E34" s="5">
+        <v>0</v>
+      </c>
+      <c r="F34" s="5">
+        <v>1</v>
+      </c>
       <c r="G34" s="5"/>
       <c r="H34" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
@@ -1974,12 +1982,16 @@
       <c r="D35" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
+      <c r="E35" s="5">
+        <v>3</v>
+      </c>
+      <c r="F35" s="5">
+        <v>0</v>
+      </c>
       <c r="G35" s="5"/>
       <c r="H35" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
@@ -1995,12 +2007,16 @@
       <c r="D36" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
+      <c r="E36" s="5">
+        <v>0</v>
+      </c>
+      <c r="F36" s="5">
+        <v>1</v>
+      </c>
       <c r="G36" s="5"/>
       <c r="H36" s="6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update forecast & dashboard 2026-06-21
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrohfm/Downloads/world-cup-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1747791C-AC36-604C-A77D-A309E88A70E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A08D16-EE24-1343-987E-C5B530BA69DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6880" yWindow="2880" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2032,12 +2032,16 @@
       <c r="D37" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
+      <c r="E37" s="5">
+        <v>5</v>
+      </c>
+      <c r="F37" s="5">
+        <v>1</v>
+      </c>
       <c r="G37" s="5"/>
       <c r="H37" s="6" t="str">
         <f t="shared" ref="H37:H68" si="1">IF(AND(ISNUMBER(E37),ISNUMBER(F37)),"entered","")</f>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
@@ -2053,12 +2057,16 @@
       <c r="D38" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
+      <c r="E38" s="5">
+        <v>2</v>
+      </c>
+      <c r="F38" s="5">
+        <v>1</v>
+      </c>
       <c r="G38" s="5"/>
       <c r="H38" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
@@ -2074,12 +2082,16 @@
       <c r="D39" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="E39" s="5"/>
-      <c r="F39" s="5"/>
+      <c r="E39" s="5">
+        <v>0</v>
+      </c>
+      <c r="F39" s="5">
+        <v>0</v>
+      </c>
       <c r="G39" s="5"/>
       <c r="H39" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
@@ -2095,12 +2107,16 @@
       <c r="D40" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
+      <c r="E40" s="5">
+        <v>0</v>
+      </c>
+      <c r="F40" s="5">
+        <v>4</v>
+      </c>
       <c r="G40" s="5"/>
       <c r="H40" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update forecast & dashboard 2026-06-22
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrohfm/Downloads/world-cup-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A08D16-EE24-1343-987E-C5B530BA69DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA002C1-CF3D-4644-8AE2-DA22180A3CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6880" yWindow="2880" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2132,12 +2132,16 @@
       <c r="D41" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
+      <c r="E41" s="5">
+        <v>4</v>
+      </c>
+      <c r="F41" s="5">
+        <v>0</v>
+      </c>
       <c r="G41" s="5"/>
       <c r="H41" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
@@ -2153,12 +2157,16 @@
       <c r="D42" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
+      <c r="E42" s="5">
+        <v>0</v>
+      </c>
+      <c r="F42" s="5">
+        <v>0</v>
+      </c>
       <c r="G42" s="5"/>
       <c r="H42" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -2174,12 +2182,16 @@
       <c r="D43" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E43" s="5"/>
-      <c r="F43" s="5"/>
+      <c r="E43" s="5">
+        <v>2</v>
+      </c>
+      <c r="F43" s="5">
+        <v>2</v>
+      </c>
       <c r="G43" s="5"/>
       <c r="H43" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -2195,12 +2207,16 @@
       <c r="D44" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
+      <c r="E44" s="5">
+        <v>1</v>
+      </c>
+      <c r="F44" s="5">
+        <v>3</v>
+      </c>
       <c r="G44" s="5"/>
       <c r="H44" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update forecast & site 2026-06-23
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrohfm/Downloads/world-cup-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA002C1-CF3D-4644-8AE2-DA22180A3CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E8C6B06-9E54-D141-B728-C8138D75E20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6880" yWindow="2880" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9300" yWindow="4500" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -2232,12 +2232,16 @@
       <c r="D45" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="E45" s="5"/>
-      <c r="F45" s="5"/>
+      <c r="E45" s="5">
+        <v>2</v>
+      </c>
+      <c r="F45" s="5">
+        <v>0</v>
+      </c>
       <c r="G45" s="5"/>
       <c r="H45" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
@@ -2253,12 +2257,16 @@
       <c r="D46" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5"/>
+      <c r="E46" s="5">
+        <v>3</v>
+      </c>
+      <c r="F46" s="5">
+        <v>0</v>
+      </c>
       <c r="G46" s="5"/>
       <c r="H46" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
@@ -2274,12 +2282,16 @@
       <c r="D47" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E47" s="5"/>
-      <c r="F47" s="5"/>
+      <c r="E47" s="5">
+        <v>3</v>
+      </c>
+      <c r="F47" s="5">
+        <v>2</v>
+      </c>
       <c r="G47" s="5"/>
       <c r="H47" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
@@ -2295,12 +2307,16 @@
       <c r="D48" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
+      <c r="E48" s="5">
+        <v>1</v>
+      </c>
+      <c r="F48" s="5">
+        <v>2</v>
+      </c>
       <c r="G48" s="5"/>
       <c r="H48" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update forecast & site 2026-06-24
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrohfm/Downloads/world-cup-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E8C6B06-9E54-D141-B728-C8138D75E20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC8CE98-9D72-E248-AE17-B55F39C3A1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9300" yWindow="4500" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2332,12 +2332,16 @@
       <c r="D49" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
+      <c r="E49" s="5">
+        <v>5</v>
+      </c>
+      <c r="F49" s="5">
+        <v>0</v>
+      </c>
       <c r="G49" s="5"/>
       <c r="H49" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
@@ -2353,12 +2357,16 @@
       <c r="D50" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E50" s="5"/>
-      <c r="F50" s="5"/>
+      <c r="E50" s="5">
+        <v>0</v>
+      </c>
+      <c r="F50" s="5">
+        <v>0</v>
+      </c>
       <c r="G50" s="5"/>
       <c r="H50" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
@@ -2374,12 +2382,16 @@
       <c r="D51" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
+      <c r="E51" s="5">
+        <v>0</v>
+      </c>
+      <c r="F51" s="5">
+        <v>1</v>
+      </c>
       <c r="G51" s="5"/>
       <c r="H51" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
@@ -2395,12 +2407,16 @@
       <c r="D52" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E52" s="5"/>
-      <c r="F52" s="5"/>
+      <c r="E52" s="5">
+        <v>1</v>
+      </c>
+      <c r="F52" s="5">
+        <v>0</v>
+      </c>
       <c r="G52" s="5"/>
       <c r="H52" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update forecast & site 2026-06-25
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrohfm/Downloads/world-cup-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC8CE98-9D72-E248-AE17-B55F39C3A1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D0AC7E0-9A10-2242-AE91-B2695C5E4EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9300" yWindow="4500" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8780" yWindow="4140" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -2432,12 +2432,16 @@
       <c r="D53" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5"/>
+      <c r="E53" s="5">
+        <v>2</v>
+      </c>
+      <c r="F53" s="5">
+        <v>1</v>
+      </c>
       <c r="G53" s="5"/>
       <c r="H53" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
@@ -2453,12 +2457,16 @@
       <c r="D54" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="E54" s="5"/>
-      <c r="F54" s="5"/>
+      <c r="E54" s="5">
+        <v>3</v>
+      </c>
+      <c r="F54" s="5">
+        <v>1</v>
+      </c>
       <c r="G54" s="5"/>
       <c r="H54" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
@@ -2474,12 +2482,16 @@
       <c r="D55" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
+      <c r="E55" s="5">
+        <v>0</v>
+      </c>
+      <c r="F55" s="5">
+        <v>3</v>
+      </c>
       <c r="G55" s="5"/>
       <c r="H55" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
@@ -2495,12 +2507,16 @@
       <c r="D56" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E56" s="5"/>
-      <c r="F56" s="5"/>
+      <c r="E56" s="5">
+        <v>4</v>
+      </c>
+      <c r="F56" s="5">
+        <v>2</v>
+      </c>
       <c r="G56" s="5"/>
       <c r="H56" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
@@ -2516,12 +2532,16 @@
       <c r="D57" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="E57" s="5"/>
-      <c r="F57" s="5"/>
+      <c r="E57" s="5">
+        <v>0</v>
+      </c>
+      <c r="F57" s="5">
+        <v>3</v>
+      </c>
       <c r="G57" s="5"/>
       <c r="H57" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
@@ -2537,12 +2557,16 @@
       <c r="D58" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="E58" s="5"/>
-      <c r="F58" s="5"/>
+      <c r="E58" s="5">
+        <v>1</v>
+      </c>
+      <c r="F58" s="5">
+        <v>0</v>
+      </c>
       <c r="G58" s="5"/>
       <c r="H58" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update forecast & site 2026-06-26
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrohfm/Downloads/world-cup-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D0AC7E0-9A10-2242-AE91-B2695C5E4EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB15F067-6A3B-E34A-9D08-59AF49CA799D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8780" yWindow="4140" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7760" yWindow="3280" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -47,6 +47,7 @@
         <r>
           <rPr>
             <sz val="10"/>
+            <color rgb="FF000000"/>
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
@@ -773,7 +774,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -810,6 +811,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -2582,12 +2589,16 @@
       <c r="D59" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="E59" s="5"/>
-      <c r="F59" s="5"/>
+      <c r="E59" s="5">
+        <v>2</v>
+      </c>
+      <c r="F59" s="5">
+        <v>1</v>
+      </c>
       <c r="G59" s="5"/>
       <c r="H59" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
@@ -2603,12 +2614,16 @@
       <c r="D60" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="E60" s="5"/>
-      <c r="F60" s="5"/>
+      <c r="E60" s="5">
+        <v>0</v>
+      </c>
+      <c r="F60" s="5">
+        <v>2</v>
+      </c>
       <c r="G60" s="5"/>
       <c r="H60" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
@@ -2624,12 +2639,16 @@
       <c r="D61" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="E61" s="5"/>
-      <c r="F61" s="5"/>
+      <c r="E61" s="5">
+        <v>1</v>
+      </c>
+      <c r="F61" s="5">
+        <v>1</v>
+      </c>
       <c r="G61" s="5"/>
       <c r="H61" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.2">
@@ -2645,12 +2664,16 @@
       <c r="D62" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
+      <c r="E62" s="5">
+        <v>1</v>
+      </c>
+      <c r="F62" s="5">
+        <v>3</v>
+      </c>
       <c r="G62" s="5"/>
       <c r="H62" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
@@ -2666,12 +2689,16 @@
       <c r="D63" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
+      <c r="E63" s="5">
+        <v>3</v>
+      </c>
+      <c r="F63" s="5">
+        <v>2</v>
+      </c>
       <c r="G63" s="5"/>
       <c r="H63" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
@@ -2687,12 +2714,16 @@
       <c r="D64" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="E64" s="5"/>
-      <c r="F64" s="5"/>
+      <c r="E64" s="5">
+        <v>0</v>
+      </c>
+      <c r="F64" s="5">
+        <v>0</v>
+      </c>
       <c r="G64" s="5"/>
       <c r="H64" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update forecast & site 2026-06-27
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrohfm/Downloads/world-cup-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB15F067-6A3B-E34A-9D08-59AF49CA799D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B31E39-3CD4-8D47-9E8A-CCA5C79879E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7760" yWindow="3280" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2739,12 +2739,16 @@
       <c r="D65" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="E65" s="5"/>
-      <c r="F65" s="5"/>
+      <c r="E65" s="5">
+        <v>1</v>
+      </c>
+      <c r="F65" s="5">
+        <v>4</v>
+      </c>
       <c r="G65" s="5"/>
       <c r="H65" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
@@ -2760,12 +2764,16 @@
       <c r="D66" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="E66" s="5"/>
-      <c r="F66" s="5"/>
+      <c r="E66" s="5">
+        <v>5</v>
+      </c>
+      <c r="F66" s="5">
+        <v>0</v>
+      </c>
       <c r="G66" s="5"/>
       <c r="H66" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
@@ -2781,12 +2789,16 @@
       <c r="D67" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="E67" s="5"/>
-      <c r="F67" s="5"/>
+      <c r="E67" s="5">
+        <v>0</v>
+      </c>
+      <c r="F67" s="5">
+        <v>0</v>
+      </c>
       <c r="G67" s="5"/>
       <c r="H67" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
@@ -2802,12 +2814,16 @@
       <c r="D68" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="E68" s="5"/>
-      <c r="F68" s="5"/>
+      <c r="E68" s="5">
+        <v>0</v>
+      </c>
+      <c r="F68" s="5">
+        <v>1</v>
+      </c>
       <c r="G68" s="5"/>
       <c r="H68" s="6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
@@ -2823,12 +2839,16 @@
       <c r="D69" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
+      <c r="E69" s="5">
+        <v>1</v>
+      </c>
+      <c r="F69" s="5">
+        <v>1</v>
+      </c>
       <c r="G69" s="5"/>
       <c r="H69" s="6" t="str">
         <f t="shared" ref="H69:H100" si="2">IF(AND(ISNUMBER(E69),ISNUMBER(F69)),"entered","")</f>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -2844,12 +2864,16 @@
       <c r="D70" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E70" s="5"/>
-      <c r="F70" s="5"/>
+      <c r="E70" s="5">
+        <v>1</v>
+      </c>
+      <c r="F70" s="5">
+        <v>5</v>
+      </c>
       <c r="G70" s="5"/>
       <c r="H70" s="6" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update forecast & site 2026-06-28
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrohfm/Downloads/world-cup-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B31E39-3CD4-8D47-9E8A-CCA5C79879E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{223C57AE-2513-274B-BADD-C7E42858EBD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7760" yWindow="3280" windowWidth="25680" windowHeight="17420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2889,12 +2889,16 @@
       <c r="D71" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="E71" s="5"/>
-      <c r="F71" s="5"/>
+      <c r="E71" s="5">
+        <v>0</v>
+      </c>
+      <c r="F71" s="5">
+        <v>2</v>
+      </c>
       <c r="G71" s="5"/>
       <c r="H71" s="6" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
@@ -2910,12 +2914,16 @@
       <c r="D72" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="E72" s="5"/>
-      <c r="F72" s="5"/>
+      <c r="E72" s="5">
+        <v>2</v>
+      </c>
+      <c r="F72" s="5">
+        <v>1</v>
+      </c>
       <c r="G72" s="5"/>
       <c r="H72" s="6" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
@@ -2931,12 +2939,16 @@
       <c r="D73" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E73" s="5"/>
-      <c r="F73" s="5"/>
+      <c r="E73" s="5">
+        <v>3</v>
+      </c>
+      <c r="F73" s="5">
+        <v>1</v>
+      </c>
       <c r="G73" s="5"/>
       <c r="H73" s="6" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.2">
@@ -2952,12 +2964,16 @@
       <c r="D74" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E74" s="5"/>
-      <c r="F74" s="5"/>
+      <c r="E74" s="5">
+        <v>0</v>
+      </c>
+      <c r="F74" s="5">
+        <v>0</v>
+      </c>
       <c r="G74" s="5"/>
       <c r="H74" s="6" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
@@ -2973,12 +2989,16 @@
       <c r="D75" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="E75" s="5"/>
-      <c r="F75" s="5"/>
+      <c r="E75" s="5">
+        <v>3</v>
+      </c>
+      <c r="F75" s="5">
+        <v>3</v>
+      </c>
       <c r="G75" s="5"/>
       <c r="H75" s="6" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
@@ -2994,12 +3014,16 @@
       <c r="D76" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="E76" s="5"/>
-      <c r="F76" s="5"/>
+      <c r="E76" s="5">
+        <v>1</v>
+      </c>
+      <c r="F76" s="5">
+        <v>3</v>
+      </c>
       <c r="G76" s="5"/>
       <c r="H76" s="6" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>entered</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update forecast & site 2026-06-29
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -2744,8 +2744,12 @@
           <t>South Africa  vs  Canada</t>
         </is>
       </c>
-      <c r="E77" s="5" t="n"/>
-      <c r="F77" s="5" t="n"/>
+      <c r="E77" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="G77" s="5" t="n"/>
       <c r="H77" s="6">
         <f>IF(AND(ISNUMBER(E77),ISNUMBER(F77)),"entered","")</f>

</xml_diff>

<commit_message>
Update forecast & site 2026-06-30
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -2829,8 +2829,12 @@
           <t>Brazil  vs  Japan</t>
         </is>
       </c>
-      <c r="E80" s="5" t="n"/>
-      <c r="F80" s="5" t="n"/>
+      <c r="E80" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F80" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="G80" s="5" t="n"/>
       <c r="H80" s="6">
         <f>IF(AND(ISNUMBER(E80),ISNUMBER(F80)),"entered","")</f>

</xml_diff>

<commit_message>
Update forecast & site 2026-07-01
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -2872,8 +2872,12 @@
           <t>France  vs  Sweden</t>
         </is>
       </c>
-      <c r="E81" s="5" t="n"/>
-      <c r="F81" s="5" t="n"/>
+      <c r="E81" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F81" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="G81" s="5" t="n"/>
       <c r="H81" s="6">
         <f>IF(AND(ISNUMBER(E81),ISNUMBER(F81)),"entered","")</f>
@@ -3197,7 +3201,7 @@
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>Winner of M74  vs  Winner of M77</t>
+          <t>Paraguay  vs  France</t>
         </is>
       </c>
       <c r="E93" s="5" t="n"/>

</xml_diff>

<commit_message>
Update forecast & site 2026-07-02
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -2996,8 +2996,12 @@
           <t>United States  vs  Bosnia &amp; Herzegovina</t>
         </is>
       </c>
-      <c r="E85" s="5" t="n"/>
-      <c r="F85" s="5" t="n"/>
+      <c r="E85" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="G85" s="5" t="n"/>
       <c r="H85" s="6">
         <f>IF(AND(ISNUMBER(E85),ISNUMBER(F85)),"entered","")</f>
@@ -3023,8 +3027,12 @@
           <t>Belgium  vs  Senegal</t>
         </is>
       </c>
-      <c r="E86" s="5" t="n"/>
-      <c r="F86" s="5" t="n"/>
+      <c r="E86" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F86" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="G86" s="5" t="n"/>
       <c r="H86" s="6">
         <f>IF(AND(ISNUMBER(E86),ISNUMBER(F86)),"entered","")</f>
@@ -3344,7 +3352,7 @@
       </c>
       <c r="D98" s="8" t="inlineStr">
         <is>
-          <t>Winner of M81  vs  Winner of M82</t>
+          <t>United States  vs  Belgium</t>
         </is>
       </c>
       <c r="E98" s="5" t="n"/>

</xml_diff>

<commit_message>
Update forecast & site 2026-07-03
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3058,8 +3058,12 @@
           <t>Portugal  vs  Croatia</t>
         </is>
       </c>
-      <c r="E87" s="5" t="n"/>
-      <c r="F87" s="5" t="n"/>
+      <c r="E87" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="G87" s="5" t="n"/>
       <c r="H87" s="6">
         <f>IF(AND(ISNUMBER(E87),ISNUMBER(F87)),"entered","")</f>
@@ -3116,8 +3120,12 @@
           <t>Switzerland  vs  Algeria</t>
         </is>
       </c>
-      <c r="E89" s="5" t="n"/>
-      <c r="F89" s="5" t="n"/>
+      <c r="E89" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F89" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="G89" s="5" t="n"/>
       <c r="H89" s="6">
         <f>IF(AND(ISNUMBER(E89),ISNUMBER(F89)),"entered","")</f>
@@ -3329,7 +3337,7 @@
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>Winner of M83  vs  Winner of M84</t>
+          <t>Portugal  vs  Spain</t>
         </is>
       </c>
       <c r="E97" s="5" t="n"/>

</xml_diff>

<commit_message>
Update forecast & site 2026-07-04
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3151,8 +3151,12 @@
           <t>Argentina  vs  Cabo Verde</t>
         </is>
       </c>
-      <c r="E90" s="5" t="n"/>
-      <c r="F90" s="5" t="n"/>
+      <c r="E90" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F90" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="G90" s="5" t="n"/>
       <c r="H90" s="6">
         <f>IF(AND(ISNUMBER(E90),ISNUMBER(F90)),"entered","")</f>
@@ -3178,8 +3182,12 @@
           <t>Colombia  vs  Ghana</t>
         </is>
       </c>
-      <c r="E91" s="5" t="n"/>
-      <c r="F91" s="5" t="n"/>
+      <c r="E91" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F91" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="G91" s="5" t="n"/>
       <c r="H91" s="6">
         <f>IF(AND(ISNUMBER(E91),ISNUMBER(F91)),"entered","")</f>
@@ -3205,9 +3213,17 @@
           <t>Australia  vs  Egypt</t>
         </is>
       </c>
-      <c r="E92" s="5" t="n"/>
-      <c r="F92" s="5" t="n"/>
-      <c r="G92" s="5" t="n"/>
+      <c r="E92" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="H92" s="6">
         <f>IF(AND(ISNUMBER(E92),ISNUMBER(F92)),"entered","")</f>
         <v/>
@@ -3391,7 +3407,7 @@
       </c>
       <c r="D99" s="8" t="inlineStr">
         <is>
-          <t>Winner of M86  vs  Winner of M88</t>
+          <t>Argentina  vs  Egypt</t>
         </is>
       </c>
       <c r="E99" s="5" t="n"/>
@@ -3418,7 +3434,7 @@
       </c>
       <c r="D100" s="8" t="inlineStr">
         <is>
-          <t>Winner of M85  vs  Winner of M87</t>
+          <t>Switzerland  vs  Colombia</t>
         </is>
       </c>
       <c r="E100" s="5" t="n"/>

</xml_diff>

<commit_message>
Update forecast & site 2026-07-05
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3248,8 +3248,12 @@
           <t>Paraguay  vs  France</t>
         </is>
       </c>
-      <c r="E93" s="5" t="n"/>
-      <c r="F93" s="5" t="n"/>
+      <c r="E93" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="G93" s="5" t="n"/>
       <c r="H93" s="6">
         <f>IF(AND(ISNUMBER(E93),ISNUMBER(F93)),"entered","")</f>
@@ -3465,7 +3469,7 @@
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>Winner of M89  vs  Winner of M90</t>
+          <t>France  vs  Morocco</t>
         </is>
       </c>
       <c r="E101" s="5" t="n"/>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-05 08:17Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="7760" yWindow="3280" windowWidth="25680" windowHeight="17420" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Index" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Team Index" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-05 11:30Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="7760" yWindow="3280" windowWidth="25680" windowHeight="17420" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Index" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Team Index" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-05 23:01Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3310,8 +3310,12 @@
           <t>Brazil  vs  Norway</t>
         </is>
       </c>
-      <c r="E95" s="5" t="n"/>
-      <c r="F95" s="5" t="n"/>
+      <c r="E95" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="G95" s="5" t="n"/>
       <c r="H95" s="6">
         <f>IF(AND(ISNUMBER(E95),ISNUMBER(F95)),"entered","")</f>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-06 03:23Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3341,8 +3341,12 @@
           <t>Mexico  vs  England</t>
         </is>
       </c>
-      <c r="E96" s="5" t="n"/>
-      <c r="F96" s="5" t="n"/>
+      <c r="E96" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F96" s="5" t="n">
+        <v>3</v>
+      </c>
       <c r="G96" s="5" t="n"/>
       <c r="H96" s="6">
         <f>IF(AND(ISNUMBER(E96),ISNUMBER(F96)),"entered","")</f>
@@ -3527,7 +3531,7 @@
       </c>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Winner of M91  vs  Winner of M92</t>
+          <t>Norway  vs  England</t>
         </is>
       </c>
       <c r="E103" s="5" t="n"/>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-06 21:28Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3372,8 +3372,12 @@
           <t>Portugal  vs  Spain</t>
         </is>
       </c>
-      <c r="E97" s="5" t="n"/>
-      <c r="F97" s="5" t="n"/>
+      <c r="E97" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="G97" s="5" t="n"/>
       <c r="H97" s="6">
         <f>IF(AND(ISNUMBER(E97),ISNUMBER(F97)),"entered","")</f>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-07 02:56Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3403,8 +3403,12 @@
           <t>United States  vs  Belgium</t>
         </is>
       </c>
-      <c r="E98" s="5" t="n"/>
-      <c r="F98" s="5" t="n"/>
+      <c r="E98" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" s="5" t="n">
+        <v>4</v>
+      </c>
       <c r="G98" s="5" t="n"/>
       <c r="H98" s="6">
         <f>IF(AND(ISNUMBER(E98),ISNUMBER(F98)),"entered","")</f>
@@ -3508,7 +3512,7 @@
       </c>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Winner of M93  vs  Winner of M94</t>
+          <t>Spain  vs  Belgium</t>
         </is>
       </c>
       <c r="E102" s="5" t="n"/>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-07 20:05Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3434,8 +3434,12 @@
           <t>Argentina  vs  Egypt</t>
         </is>
       </c>
-      <c r="E99" s="5" t="n"/>
-      <c r="F99" s="5" t="n"/>
+      <c r="E99" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F99" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="G99" s="5" t="n"/>
       <c r="H99" s="6">
         <f>IF(AND(ISNUMBER(E99),ISNUMBER(F99)),"entered","")</f>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-07 23:01Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3465,8 +3465,12 @@
           <t>Switzerland  vs  Colombia</t>
         </is>
       </c>
-      <c r="E100" s="5" t="n"/>
-      <c r="F100" s="5" t="n"/>
+      <c r="E100" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F100" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="G100" s="5" t="n"/>
       <c r="H100" s="6">
         <f>IF(AND(ISNUMBER(E100),ISNUMBER(F100)),"entered","")</f>
@@ -3570,7 +3574,7 @@
       </c>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Winner of M95  vs  Winner of M96</t>
+          <t>Argentina  vs  Switzerland</t>
         </is>
       </c>
       <c r="E104" s="5" t="n"/>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-09 23:10Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3496,8 +3496,12 @@
           <t>France  vs  Morocco</t>
         </is>
       </c>
-      <c r="E101" s="5" t="n"/>
-      <c r="F101" s="5" t="n"/>
+      <c r="E101" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F101" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="G101" s="5" t="n"/>
       <c r="H101" s="6">
         <f>IF(AND(ISNUMBER(E101),ISNUMBER(F101)),"entered","")</f>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-10 22:59Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3527,8 +3527,12 @@
           <t>Spain  vs  Belgium</t>
         </is>
       </c>
-      <c r="E102" s="5" t="n"/>
-      <c r="F102" s="5" t="n"/>
+      <c r="E102" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F102" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="G102" s="5" t="n"/>
       <c r="H102" s="6">
         <f>IF(AND(ISNUMBER(E102),ISNUMBER(F102)),"entered","")</f>
@@ -3605,7 +3609,7 @@
       </c>
       <c r="D105" s="8" t="inlineStr">
         <is>
-          <t>Winner of M97  vs  Winner of M98</t>
+          <t>France  vs  Spain</t>
         </is>
       </c>
       <c r="E105" s="5" t="n"/>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-12 02:36Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3558,8 +3558,12 @@
           <t>Norway  vs  England</t>
         </is>
       </c>
-      <c r="E103" s="5" t="n"/>
-      <c r="F103" s="5" t="n"/>
+      <c r="E103" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F103" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="G103" s="5" t="n"/>
       <c r="H103" s="6">
         <f>IF(AND(ISNUMBER(E103),ISNUMBER(F103)),"entered","")</f>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-12 06:32Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3589,8 +3589,12 @@
           <t>Argentina  vs  Switzerland</t>
         </is>
       </c>
-      <c r="E104" s="5" t="n"/>
-      <c r="F104" s="5" t="n"/>
+      <c r="E104" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F104" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="G104" s="5" t="n"/>
       <c r="H104" s="6">
         <f>IF(AND(ISNUMBER(E104),ISNUMBER(F104)),"entered","")</f>
@@ -3640,7 +3644,7 @@
       </c>
       <c r="D106" s="8" t="inlineStr">
         <is>
-          <t>Winner of M99  vs  Winner of M100</t>
+          <t>England  vs  Argentina</t>
         </is>
       </c>
       <c r="E106" s="5" t="n"/>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-14 22:56Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3620,8 +3620,12 @@
           <t>France  vs  Spain</t>
         </is>
       </c>
-      <c r="E105" s="5" t="n"/>
-      <c r="F105" s="5" t="n"/>
+      <c r="E105" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="G105" s="5" t="n"/>
       <c r="H105" s="6">
         <f>IF(AND(ISNUMBER(E105),ISNUMBER(F105)),"entered","")</f>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-15 22:58Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3651,8 +3651,12 @@
           <t>England  vs  Argentina</t>
         </is>
       </c>
-      <c r="E106" s="5" t="n"/>
-      <c r="F106" s="5" t="n"/>
+      <c r="E106" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F106" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="G106" s="5" t="n"/>
       <c r="H106" s="6">
         <f>IF(AND(ISNUMBER(E106),ISNUMBER(F106)),"entered","")</f>
@@ -3675,7 +3679,7 @@
       </c>
       <c r="D107" s="8" t="inlineStr">
         <is>
-          <t>Loser of M101  vs  Loser of M102</t>
+          <t>France  vs  England</t>
         </is>
       </c>
       <c r="E107" s="5" t="n"/>
@@ -3702,7 +3706,7 @@
       </c>
       <c r="D108" s="8" t="inlineStr">
         <is>
-          <t>Winner of M101  vs  Winner of M102</t>
+          <t>Spain  vs  Argentina</t>
         </is>
       </c>
       <c r="E108" s="5" t="n"/>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-19 02:33Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3682,8 +3682,12 @@
           <t>France  vs  England</t>
         </is>
       </c>
-      <c r="E107" s="5" t="n"/>
-      <c r="F107" s="5" t="n"/>
+      <c r="E107" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F107" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="G107" s="5" t="n"/>
       <c r="H107" s="6">
         <f>IF(AND(ISNUMBER(E107),ISNUMBER(F107)),"entered","")</f>

</xml_diff>

<commit_message>
Auto snapshot 2026-07-19 22:50Z
</commit_message>
<xml_diff>
--- a/wc2026_results.xlsx
+++ b/wc2026_results.xlsx
@@ -3713,8 +3713,12 @@
           <t>Spain  vs  Argentina</t>
         </is>
       </c>
-      <c r="E108" s="5" t="n"/>
-      <c r="F108" s="5" t="n"/>
+      <c r="E108" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="G108" s="5" t="n"/>
       <c r="H108" s="6">
         <f>IF(AND(ISNUMBER(E108),ISNUMBER(F108)),"entered","")</f>

</xml_diff>